<commit_message>
Remove internal GitHub Actions cron schedule in favor of cron-job.org
</commit_message>
<xml_diff>
--- a/data/restaurant_ratings.xlsx
+++ b/data/restaurant_ratings.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Daily Ratings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Ratings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1186,43 +1186,6 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>2 Oct</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n">
-        <v>144</v>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>231</v>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F20" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H20" s="4" t="n">
-        <v>74</v>
-      </c>
-      <c r="I20" s="5" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="J20" s="4" t="n">
-        <v>52</v>
-      </c>
-      <c r="K20" s="5" t="n">
-        <v>3.7</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:A3"/>

</xml_diff>

<commit_message>
Match Excel tracker and email table styling with reference design
</commit_message>
<xml_diff>
--- a/data/restaurant_ratings.xlsx
+++ b/data/restaurant_ratings.xlsx
@@ -28,19 +28,19 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Arial"/>
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
@@ -54,12 +54,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8F9FA"/>
-        <bgColor rgb="00F8F9FA"/>
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -81,26 +81,43 @@
         <color rgb="00D3D3D3"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="007F7F7F"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -470,719 +487,719 @@
   <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13.5" customWidth="1" min="1" max="1"/>
+    <col width="11.5" customWidth="1" min="2" max="2"/>
+    <col width="10.5" customWidth="1" min="3" max="3"/>
+    <col width="11.5" customWidth="1" min="4" max="4"/>
+    <col width="10.5" customWidth="1" min="5" max="5"/>
+    <col width="11.5" customWidth="1" min="6" max="6"/>
+    <col width="10.5" customWidth="1" min="7" max="7"/>
+    <col width="11.5" customWidth="1" min="8" max="8"/>
+    <col width="10.5" customWidth="1" min="9" max="9"/>
+    <col width="11.5" customWidth="1" min="10" max="10"/>
+    <col width="10.5" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Kiplings</t>
         </is>
       </c>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Casa Loco Express</t>
         </is>
       </c>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="1" t="n"/>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Google</t>
         </is>
       </c>
-      <c r="C2" s="1" t="n"/>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Zomato</t>
         </is>
       </c>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Google</t>
         </is>
       </c>
-      <c r="G2" s="1" t="n"/>
-      <c r="H2" s="1" t="inlineStr">
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Zomato - Delivery</t>
         </is>
       </c>
-      <c r="I2" s="1" t="n"/>
-      <c r="J2" s="1" t="inlineStr">
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Swiggy - Delivery</t>
         </is>
       </c>
-      <c r="K2" s="1" t="n"/>
-    </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="K2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Total no</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Total no</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Total no</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Total no</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Total no</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>15 Sept</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="5" t="n">
         <v>116</v>
       </c>
-      <c r="C4" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="C4" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>153</v>
       </c>
-      <c r="E4" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H4" s="4" t="n">
+      <c r="E4" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" s="5" t="n">
         <v>63</v>
       </c>
-      <c r="I4" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J4" s="4" t="n">
+      <c r="I4" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J4" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="K4" s="6" t="n">
         <v>3.8</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>16 Sept</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="5" t="n">
         <v>121</v>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="D5" s="4" t="n">
+      <c r="C5" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D5" s="5" t="n">
         <v>158</v>
       </c>
-      <c r="E5" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H5" s="4" t="n">
+      <c r="E5" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="5" t="n">
         <v>63</v>
       </c>
-      <c r="I5" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J5" s="4" t="n">
+      <c r="I5" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J5" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="K5" s="5" t="n">
+      <c r="K5" s="6" t="n">
         <v>3.8</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>17 Sept</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="5" t="n">
         <v>121</v>
       </c>
-      <c r="C6" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="D6" s="4" t="n">
+      <c r="C6" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D6" s="5" t="n">
         <v>164</v>
       </c>
-      <c r="E6" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H6" s="4" t="n">
+      <c r="E6" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>65</v>
       </c>
-      <c r="I6" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J6" s="4" t="n">
+      <c r="I6" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J6" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="K6" s="5" t="n">
+      <c r="K6" s="6" t="n">
         <v>3.8</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>18 Sept</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="5" t="n">
         <v>120</v>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="D7" s="4" t="n">
+      <c r="C7" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D7" s="5" t="n">
         <v>166</v>
       </c>
-      <c r="E7" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H7" s="4" t="n">
+      <c r="E7" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>66</v>
       </c>
-      <c r="I7" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J7" s="4" t="n">
+      <c r="I7" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J7" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="K7" s="5" t="n">
+      <c r="K7" s="6" t="n">
         <v>3.8</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>19 Sept</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="5" t="n">
         <v>121</v>
       </c>
-      <c r="C8" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="D8" s="4" t="n">
+      <c r="C8" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D8" s="5" t="n">
         <v>171</v>
       </c>
-      <c r="E8" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H8" s="4" t="n">
+      <c r="E8" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>67</v>
       </c>
-      <c r="I8" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J8" s="4" t="n">
+      <c r="I8" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J8" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="K8" s="6" t="n">
         <v>3.8</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>20 Sept</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="5" t="n">
         <v>121</v>
       </c>
-      <c r="C9" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="D9" s="4" t="n">
+      <c r="C9" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D9" s="5" t="n">
         <v>178</v>
       </c>
-      <c r="E9" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H9" s="4" t="n">
+      <c r="E9" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" s="5" t="n">
         <v>67</v>
       </c>
-      <c r="I9" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J9" s="4" t="n">
+      <c r="I9" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J9" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="K9" s="5" t="n">
+      <c r="K9" s="6" t="n">
         <v>3.8</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>21 Sept</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="5" t="n">
         <v>123</v>
       </c>
-      <c r="C10" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="D10" s="4" t="n">
+      <c r="C10" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D10" s="5" t="n">
         <v>187</v>
       </c>
-      <c r="E10" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H10" s="4" t="n">
+      <c r="E10" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" s="5" t="n">
         <v>67</v>
       </c>
-      <c r="I10" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J10" s="4" t="n">
+      <c r="I10" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J10" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="K10" s="5" t="n">
+      <c r="K10" s="6" t="n">
         <v>3.8</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>22 Sept</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="5" t="n">
         <v>124</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="5" t="n">
         <v>192</v>
       </c>
-      <c r="E11" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H11" s="4" t="n">
+      <c r="E11" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" s="5" t="n">
         <v>68</v>
       </c>
-      <c r="I11" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J11" s="4" t="n">
+      <c r="I11" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J11" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="K11" s="5" t="n">
+      <c r="K11" s="6" t="n">
         <v>3.8</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>23 Sept</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="5" t="n">
         <v>125</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="5" t="n">
         <v>194</v>
       </c>
-      <c r="E12" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H12" s="4" t="n">
+      <c r="E12" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" s="5" t="n">
         <v>68</v>
       </c>
-      <c r="I12" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J12" s="4" t="n">
+      <c r="I12" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J12" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="K12" s="5" t="n">
+      <c r="K12" s="6" t="n">
         <v>3.8</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>24 Sept</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="5" t="n">
         <v>124</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="5" t="n">
         <v>198</v>
       </c>
-      <c r="E13" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="F13" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H13" s="4" t="n">
+      <c r="E13" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H13" s="5" t="n">
         <v>70</v>
       </c>
-      <c r="I13" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J13" s="4" t="n">
+      <c r="I13" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J13" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="K13" s="5" t="n">
+      <c r="K13" s="6" t="n">
         <v>3.8</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>25 Sept</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="5" t="n">
         <v>129</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="E14" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G14" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H14" s="4" t="n">
+      <c r="E14" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H14" s="5" t="n">
         <v>71</v>
       </c>
-      <c r="I14" s="5" t="n">
+      <c r="I14" s="6" t="n">
         <v>4.2</v>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="J14" s="5" t="n">
         <v>47</v>
       </c>
-      <c r="K14" s="5" t="n">
+      <c r="K14" s="6" t="n">
         <v>3.8</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>27 Sept</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="5" t="n">
         <v>142</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="5" t="n">
         <v>217</v>
       </c>
-      <c r="E15" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H15" s="4" t="n">
+      <c r="E15" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H15" s="5" t="n">
         <v>73</v>
       </c>
-      <c r="I15" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J15" s="4" t="n">
+      <c r="I15" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J15" s="5" t="n">
         <v>47</v>
       </c>
-      <c r="K15" s="5" t="n">
+      <c r="K15" s="6" t="n">
         <v>3.8</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>28 Sept</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B16" s="5" t="n">
         <v>143</v>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C16" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D16" s="5" t="n">
         <v>222</v>
       </c>
-      <c r="E16" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H16" s="4" t="n">
+      <c r="E16" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H16" s="5" t="n">
         <v>73</v>
       </c>
-      <c r="I16" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J16" s="4" t="n">
+      <c r="I16" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J16" s="5" t="n">
         <v>48</v>
       </c>
-      <c r="K16" s="5" t="n">
+      <c r="K16" s="6" t="n">
         <v>3.7</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>29 Sept</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n">
+      <c r="B17" s="5" t="n">
         <v>143</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" s="5" t="n">
         <v>225</v>
       </c>
-      <c r="E17" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G17" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H17" s="4" t="n">
+      <c r="E17" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>73</v>
       </c>
-      <c r="I17" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J17" s="4" t="n">
+      <c r="I17" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J17" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="K17" s="5" t="n">
+      <c r="K17" s="6" t="n">
         <v>3.7</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>30 Sept</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n">
+      <c r="B18" s="5" t="n">
         <v>143</v>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C18" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="D18" s="5" t="n">
         <v>229</v>
       </c>
-      <c r="E18" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F18" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H18" s="4" t="n">
+      <c r="E18" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" s="5" t="n">
         <v>73</v>
       </c>
-      <c r="I18" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="J18" s="4" t="n">
+      <c r="I18" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J18" s="5" t="n">
         <v>52</v>
       </c>
-      <c r="K18" s="5" t="n">
+      <c r="K18" s="6" t="n">
         <v>3.7</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>1 Oct</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n">
-        <v>143</v>
-      </c>
-      <c r="C19" s="5" t="n">
+      <c r="B19" s="5" t="n">
+        <v>144</v>
+      </c>
+      <c r="C19" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="D19" s="5" t="n">
         <v>231</v>
       </c>
-      <c r="E19" s="5" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F19" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H19" s="4" t="n">
+      <c r="E19" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H19" s="5" t="n">
         <v>74</v>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="I19" s="6" t="n">
         <v>4.2</v>
       </c>
-      <c r="J19" s="4" t="n">
+      <c r="J19" s="5" t="n">
         <v>52</v>
       </c>
-      <c r="K19" s="5" t="n">
+      <c r="K19" s="6" t="n">
         <v>3.7</v>
       </c>
     </row>

</xml_diff>